<commit_message>
Documento y graficos modificados
</commit_message>
<xml_diff>
--- a/Graficos.xlsx
+++ b/Graficos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://estudianteccr-my.sharepoint.com/personal/f_vargas_1_estudiantec_cr/Documents/III Semestre/Análisis de algoritmos/Analisis - Proyecto 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salas\Dev\Tec\Analisis_algoritmos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="353" documentId="8_{2FCCCEEF-840E-4E86-ADF0-9A2D3957909A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CF8ACC2-FB22-4CB6-817C-81339704D792}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C34DCDD2-F293-426B-8C74-35D9DD32C06F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="738" firstSheet="1" activeTab="2" xr2:uid="{E6716E66-8208-44B0-BF49-B934528B8CBC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="738" activeTab="1" xr2:uid="{E6716E66-8208-44B0-BF49-B934528B8CBC}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="9" r:id="rId1"/>
@@ -185,9 +185,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -197,10 +194,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -400,28 +400,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>862</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10543</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>147706</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2519139</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>52013537</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1232434812</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>31697270344</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -622,28 +622,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>1238</c:v>
+                  <c:v>1211</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10732</c:v>
+                  <c:v>10876</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>82280</c:v>
+                  <c:v>82159</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>659981</c:v>
+                  <c:v>660538</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5601977</c:v>
+                  <c:v>5601086</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>49018284</c:v>
+                  <c:v>49009340</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>447045794</c:v>
+                  <c:v>447043296</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4134934663</c:v>
+                  <c:v>4134903008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1174,28 +1174,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>862</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10543</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>147706</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2519139</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>52013537</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1232434812</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>31697270344</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1396,28 +1396,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>1238</c:v>
+                  <c:v>1211</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10732</c:v>
+                  <c:v>10876</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>82280</c:v>
+                  <c:v>82159</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>659981</c:v>
+                  <c:v>660538</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5601977</c:v>
+                  <c:v>5601086</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>49018284</c:v>
+                  <c:v>49009340</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>447045794</c:v>
+                  <c:v>447043296</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4134934663</c:v>
+                  <c:v>4134903008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1950,28 +1950,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>862</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10543</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>147706</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2519139</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>52013537</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1232434812</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>31697270344</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2172,28 +2172,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>1238</c:v>
+                  <c:v>1211</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10732</c:v>
+                  <c:v>10876</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>82280</c:v>
+                  <c:v>82159</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>659981</c:v>
+                  <c:v>660538</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5601977</c:v>
+                  <c:v>5601086</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>49018284</c:v>
+                  <c:v>49009340</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>447045794</c:v>
+                  <c:v>447043296</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4134934663</c:v>
+                  <c:v>4134903008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2590,7 +2590,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.15035676739660456"/>
+          <c:y val="0.16841080476569795"/>
+          <c:w val="0.76596150762733628"/>
+          <c:h val="0.72661841952843564"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -2619,7 +2629,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="8"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -2672,28 +2682,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>69</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>862</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>10543</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>147706</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2519139</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>52013537</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1232434812</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>31697270344</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2784,6 +2794,7 @@
         <c:axId val="1253043247"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="10"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2962,7 +2973,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="9"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -3127,6 +3138,7 @@
         <c:axId val="1651876879"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="10"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -3305,7 +3317,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="9"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -3358,28 +3370,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>1238</c:v>
+                  <c:v>1211</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10732</c:v>
+                  <c:v>10876</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>82280</c:v>
+                  <c:v>82159</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>659981</c:v>
+                  <c:v>660538</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5601977</c:v>
+                  <c:v>5601086</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>49018284</c:v>
+                  <c:v>49009340</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>447045794</c:v>
+                  <c:v>447043296</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4134934663</c:v>
+                  <c:v>4134903008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3648,7 +3660,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:size val="9"/>
             <c:spPr>
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
@@ -3813,6 +3825,7 @@
         <c:axId val="197398416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="10"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -7925,7 +7938,7 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>576594</xdr:colOff>
+      <xdr:colOff>365760</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>123876</xdr:rowOff>
     </xdr:from>
@@ -8069,10 +8082,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_2" connectionId="3" xr16:uid="{CA9057C4-CDDB-4F57-A2C5-4356494F2382}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="7">
@@ -8184,7 +8193,7 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{676D18AF-8132-42D7-81E5-FEC1F6996AB9}" name="Tamaño"/>
     <tableColumn id="2" xr3:uid="{12EAA182-9A8F-49A3-8410-CD053F604826}" name="Divisibilidad">
-      <calculatedColumnFormula>INDEX(Resultados_1_Divisi_n_por_tenta!#REF!,MATCH(Graficos!A2,Resultados_1_Divisi_n_por_tenta!A2:A9,0))</calculatedColumnFormula>
+      <calculatedColumnFormula>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A2,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{5D5B113E-B30D-4469-BBE8-8083191C2CD9}" name="Eratóstenes">
       <calculatedColumnFormula>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A2,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</calculatedColumnFormula>
@@ -8990,9 +8999,9 @@
       <c r="A2">
         <v>10</v>
       </c>
-      <c r="B2" t="e">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!#REF!,MATCH(Graficos!A2,Resultados_1_Divisi_n_por_tenta!A2:A9,0))</f>
-        <v>#REF!</v>
+      <c r="B2">
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A2,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>69</v>
       </c>
       <c r="C2">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A2,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9000,7 +9009,7 @@
       </c>
       <c r="D2">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A2,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>1238</v>
+        <v>1211</v>
       </c>
       <c r="E2">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A2,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9012,8 +9021,8 @@
         <v>100</v>
       </c>
       <c r="B3">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D10,MATCH(Graficos!A3,Resultados_1_Divisi_n_por_tenta!A3:A10,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A3,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>862</v>
       </c>
       <c r="C3">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A3,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9021,7 +9030,7 @@
       </c>
       <c r="D3">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A3,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>10732</v>
+        <v>10876</v>
       </c>
       <c r="E3">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A3,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9033,8 +9042,8 @@
         <v>1000</v>
       </c>
       <c r="B4">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D11,MATCH(Graficos!A4,Resultados_1_Divisi_n_por_tenta!A4:A11,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A4,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>10543</v>
       </c>
       <c r="C4">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A4,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9042,7 +9051,7 @@
       </c>
       <c r="D4">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A4,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>82280</v>
+        <v>82159</v>
       </c>
       <c r="E4">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A4,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9054,8 +9063,8 @@
         <v>10000</v>
       </c>
       <c r="B5">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D12,MATCH(Graficos!A5,Resultados_1_Divisi_n_por_tenta!A5:A12,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A5,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>147706</v>
       </c>
       <c r="C5">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A5,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9063,7 +9072,7 @@
       </c>
       <c r="D5">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A5,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>659981</v>
+        <v>660538</v>
       </c>
       <c r="E5">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A5,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9075,8 +9084,8 @@
         <v>100000</v>
       </c>
       <c r="B6">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D13,MATCH(Graficos!A6,Resultados_1_Divisi_n_por_tenta!A6:A13,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A6,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>2519139</v>
       </c>
       <c r="C6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A6,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9084,7 +9093,7 @@
       </c>
       <c r="D6">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A6,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>5601977</v>
+        <v>5601086</v>
       </c>
       <c r="E6">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A6,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9096,8 +9105,8 @@
         <v>1000000</v>
       </c>
       <c r="B7">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D14,MATCH(Graficos!A7,Resultados_1_Divisi_n_por_tenta!A7:A14,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A7,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>52013537</v>
       </c>
       <c r="C7">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A7,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9105,7 +9114,7 @@
       </c>
       <c r="D7">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A7,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>49018284</v>
+        <v>49009340</v>
       </c>
       <c r="E7">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A7,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9117,8 +9126,8 @@
         <v>10000000</v>
       </c>
       <c r="B8">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D15,MATCH(Graficos!A8,Resultados_1_Divisi_n_por_tenta!A8:A15,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A8,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>1232434812</v>
       </c>
       <c r="C8">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A8,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9126,7 +9135,7 @@
       </c>
       <c r="D8">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A8,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>447045794</v>
+        <v>447043296</v>
       </c>
       <c r="E8">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A8,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9138,8 +9147,8 @@
         <v>100000000</v>
       </c>
       <c r="B9">
-        <f>INDEX(Resultados_1_Divisi_n_por_tenta!D10:D16,MATCH(Graficos!A9,Resultados_1_Divisi_n_por_tenta!A9:A16,0))</f>
-        <v>0</v>
+        <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[Líneas ejecutadas],MATCH(A9,Resultados_1_Divisi_n_por_tentativa_optimizado[Tamaño],0))</f>
+        <v>31697270344</v>
       </c>
       <c r="C9">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A9,Resultados_2_Criba_de_Erat_stenes[Tamaño],0))</f>
@@ -9147,7 +9156,7 @@
       </c>
       <c r="D9">
         <f>INDEX(Resultados_4_Miller_Rabin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A9,Resultados_4_Miller_Rabin[Tamaño],0))</f>
-        <v>4134934663</v>
+        <v>4134903008</v>
       </c>
       <c r="E9">
         <f>INDEX(Resultados_3_Criba_de_Atkin[Cantidad de líneas ejecutadas (Suma asig + comp)],MATCH(A9,Resultados_3_Criba_de_Atkin[Tamaño],0))</f>
@@ -9185,603 +9194,603 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="I1" s="7" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="I1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
     </row>
     <row r="2" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="2"/>
-      <c r="K2" s="3" t="s">
+      <c r="J2" s="7"/>
+      <c r="K2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>10</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>100</v>
       </c>
       <c r="C3">
         <f>B3/A3</f>
         <v>10</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>10.8125</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>13</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>12.492753623188406</v>
       </c>
-      <c r="G3" s="8" t="e">
+      <c r="G3" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A3,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I3" s="3">
+        <v>0.62172284644194753</v>
+      </c>
+      <c r="I3" s="2">
         <v>10</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="2">
         <v>100</v>
       </c>
       <c r="K3">
         <f>J3/I3</f>
         <v>10</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($J3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($I3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.9375</v>
       </c>
-      <c r="M3" s="8">
+      <c r="M3" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.516129032258064</v>
       </c>
-      <c r="N3" s="8">
+      <c r="N3" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.730158730158729</v>
       </c>
-      <c r="O3" s="8" t="e">
+      <c r="O3" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I3,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>1.0293255131964809</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>1000</v>
       </c>
       <c r="C4">
         <f t="shared" ref="C4:C12" si="0">B4/A4</f>
         <v>100</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>131.0625</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>159.35849056603774</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>152.79710144927537</v>
       </c>
-      <c r="G4" s="8" t="e">
+      <c r="G4" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A4,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I4" s="3">
+        <v>5.7116104868913853</v>
+      </c>
+      <c r="I4" s="2">
         <v>10</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="2">
         <v>1000</v>
       </c>
       <c r="K4">
         <f t="shared" ref="K4:K12" si="1">J4/I4</f>
         <v>100</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>126.09375</v>
       </c>
-      <c r="M4" s="8">
+      <c r="M4" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>112.3225806451613</v>
       </c>
-      <c r="N4" s="8">
+      <c r="N4" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>119.31746031746032</v>
       </c>
-      <c r="O4" s="8" t="e">
+      <c r="O4" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I4,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>5.1466275659824046</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>10</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>10000</v>
       </c>
       <c r="C5">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>1935.25</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>2202.6792452830186</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>2140.6666666666665</v>
       </c>
-      <c r="G5" s="8" t="e">
+      <c r="G5" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A5,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I5" s="3">
+        <v>26.337078651685392</v>
+      </c>
+      <c r="I5" s="2">
         <v>10</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="2">
         <v>10000</v>
       </c>
       <c r="K5">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>1416.21875</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>1200.1290322580646</v>
       </c>
-      <c r="N5" s="8">
+      <c r="N5" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>1309.8888888888889</v>
       </c>
-      <c r="O5" s="8" t="e">
+      <c r="O5" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I5,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>29.354838709677416</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>10</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>100000</v>
       </c>
       <c r="C6">
         <f t="shared" si="0"/>
         <v>10000</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>35423.5</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>36837.037735849059</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>36509.260869565216</v>
       </c>
-      <c r="G6" s="8" t="e">
+      <c r="G6" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A6,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I6" s="3">
+        <v>166.72284644194755</v>
+      </c>
+      <c r="I6" s="2">
         <v>10</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>100000</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>15504.125</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>12702.354838709678</v>
       </c>
-      <c r="N6" s="8">
+      <c r="N6" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>14125.476190476191</v>
       </c>
-      <c r="O6" s="8" t="e">
+      <c r="O6" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I6,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>110.3108504398827</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>100</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>1000</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>12.121387283236995</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>12.258345428156749</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>12.230858468677495</v>
       </c>
-      <c r="G7" s="8" t="e">
+      <c r="G7" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A7,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I7" s="3">
+        <v>9.1867469879518069</v>
+      </c>
+      <c r="I7" s="2">
         <v>100</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="2">
         <v>1000</v>
       </c>
       <c r="K7">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>11.528571428571428</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.680981595092025</v>
       </c>
-      <c r="N7" s="8">
+      <c r="N7" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>11.1198224852071</v>
       </c>
-      <c r="O7" s="8" t="e">
+      <c r="O7" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I7,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>1000</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>10000</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>14.765855984740105</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>13.822164338148236</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>14.009864364981505</v>
       </c>
-      <c r="G8" s="8" t="e">
+      <c r="G8" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A8,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I8" s="3">
+        <v>4.6111475409836071</v>
+      </c>
+      <c r="I8" s="2">
         <v>1000</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <v>10000</v>
       </c>
       <c r="K8">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>11.231474597273854</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.684663986214819</v>
       </c>
-      <c r="N8" s="8">
+      <c r="N8" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.978182785685778</v>
       </c>
-      <c r="O8" s="8" t="e">
+      <c r="O8" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I8,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>5.7037037037037033</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>100000</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>1000000</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>21.79257413863678</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>20.314884578328929</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>20.647346970532393</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A9,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>9.1428571428571423</v>
+        <v>8.3461305178029868</v>
       </c>
       <c r="I9" s="1">
         <v>100000</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>1000000</v>
       </c>
       <c r="K9">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.730541468802658</v>
       </c>
-      <c r="M9" s="8">
+      <c r="M9" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.473582495498675</v>
       </c>
-      <c r="N9" s="8">
+      <c r="N9" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.616839999775257</v>
       </c>
-      <c r="O9" s="8">
+      <c r="O9" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I9,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>1.9090909090909092</v>
+        <v>4.0236601446193108</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="5">
+      <c r="A10" s="4">
         <v>1000000</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>10000000</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>24.405070862602365</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>23.473216259309375</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>23.694501144961553</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A10,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>24.65625</v>
-      </c>
-      <c r="I10" s="5">
+        <v>25.006104519713183</v>
+      </c>
+      <c r="I10" s="4">
         <v>1000000</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <v>10000000</v>
       </c>
       <c r="K10">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L10" s="8">
+      <c r="L10" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.588050374124327</v>
       </c>
-      <c r="M10" s="8">
+      <c r="M10" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.391511934152787</v>
       </c>
-      <c r="N10" s="8">
+      <c r="N10" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>10.502257784442577</v>
       </c>
-      <c r="O10" s="8">
+      <c r="O10" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I10,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>5.8095238095238093</v>
+        <v>4.5928419466945041</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>100</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>10000</v>
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>178.98265895953756</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>169.43686502177067</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>171.35266821345706</v>
       </c>
-      <c r="G11" s="8" t="e">
+      <c r="G11" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A11,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>42.361445783132531</v>
       </c>
       <c r="I11" s="1">
         <v>100</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="4">
         <v>10000</v>
       </c>
       <c r="K11">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>129.48285714285714</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>114.12269938650307</v>
       </c>
-      <c r="N11" s="8">
+      <c r="N11" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>122.07544378698225</v>
       </c>
-      <c r="O11" s="8" t="e">
+      <c r="O11" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I11,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>28.518518518518515</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1000</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>100000</v>
       </c>
       <c r="C12">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($B12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Asignaciones]],MATCH($A12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>270.27944682880303</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($B12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Comparaciones]],MATCH($A12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>231.15829978688137</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($B12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Líneas ejecutadas]],MATCH($A12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
         <v>238.93948591482501</v>
       </c>
-      <c r="G12" s="8" t="e">
+      <c r="G12" s="6">
         <f>INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($B12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))/INDEX(Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tiempo de ejecución (ms)]],MATCH($A12,Resultados_1_Divisi_n_por_tentativa_optimizado[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>29.190163934426231</v>
       </c>
       <c r="I12" s="1">
         <v>1000</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="4">
         <v>100000</v>
       </c>
       <c r="K12">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($B12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Asignaciones]],MATCH($A12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>122.95712515489467</v>
       </c>
-      <c r="M12" s="8">
+      <c r="M12" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($J12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Comparaciones]],MATCH($I12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>113.08816771970132</v>
       </c>
-      <c r="N12" s="8">
+      <c r="N12" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($J12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Cantidad de líneas ejecutadas (Suma asig + comp)]],MATCH($I12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
         <v>118.38565917254223</v>
       </c>
-      <c r="O12" s="8" t="e">
+      <c r="O12" s="6">
         <f>INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($J12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))/INDEX(Resultados_2_Criba_de_Erat_stenes[[#All],[Tiempo de ejecución (ms)]],MATCH($I12,Resultados_2_Criba_de_Erat_stenes[[#All],[Tamaño]],0))</f>
-        <v>#DIV/0!</v>
+        <v>21.433618233618237</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -9847,7 +9856,7 @@
         <v>69</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>2.6700000000000002E-2</v>
       </c>
       <c r="F2">
         <v>15</v>
@@ -9867,7 +9876,7 @@
         <v>862</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1.66E-2</v>
       </c>
       <c r="F3">
         <v>15</v>
@@ -9887,7 +9896,7 @@
         <v>10543</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.1525</v>
       </c>
       <c r="F4">
         <v>15</v>
@@ -9907,7 +9916,7 @@
         <v>147706</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0.70320000000000005</v>
       </c>
       <c r="F5">
         <v>15</v>
@@ -9927,7 +9936,7 @@
         <v>2519139</v>
       </c>
       <c r="E6">
-        <v>7</v>
+        <v>4.4515000000000002</v>
       </c>
       <c r="F6">
         <v>15</v>
@@ -9947,7 +9956,7 @@
         <v>52013537</v>
       </c>
       <c r="E7">
-        <v>64</v>
+        <v>37.152799999999999</v>
       </c>
       <c r="F7">
         <v>15</v>
@@ -9967,7 +9976,7 @@
         <v>1232434812</v>
       </c>
       <c r="E8">
-        <v>1578</v>
+        <v>929.04679999999996</v>
       </c>
       <c r="F8">
         <v>15</v>
@@ -9987,7 +9996,7 @@
         <v>31697270344</v>
       </c>
       <c r="E9">
-        <v>38306</v>
+        <v>22792.6158</v>
       </c>
       <c r="F9">
         <v>15</v>
@@ -10048,7 +10057,7 @@
         <v>63</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="F2">
         <v>11</v>
@@ -10068,7 +10077,7 @@
         <v>676</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>3.5099999999999999E-2</v>
       </c>
       <c r="F3">
         <v>11</v>
@@ -10088,7 +10097,7 @@
         <v>7517</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.17549999999999999</v>
       </c>
       <c r="F4">
         <v>11</v>
@@ -10108,7 +10117,7 @@
         <v>82523</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>1.0009999999999999</v>
       </c>
       <c r="F5">
         <v>11</v>
@@ -10128,7 +10137,7 @@
         <v>889905</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>3.7616000000000001</v>
       </c>
       <c r="F6">
         <v>11</v>
@@ -10148,7 +10157,7 @@
         <v>9447979</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>15.135400000000001</v>
       </c>
       <c r="F7">
         <v>11</v>
@@ -10168,7 +10177,7 @@
         <v>99225111</v>
       </c>
       <c r="E8">
-        <v>122</v>
+        <v>69.514499999999998</v>
       </c>
       <c r="F8">
         <v>11</v>
@@ -10188,7 +10197,7 @@
         <v>1033504526</v>
       </c>
       <c r="E9">
-        <v>1454</v>
+        <v>1362.2035000000001</v>
       </c>
       <c r="F9">
         <v>11</v>
@@ -10249,7 +10258,7 @@
         <v>172</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>3.7600000000000001E-2</v>
       </c>
       <c r="F2">
         <v>30</v>
@@ -10269,7 +10278,7 @@
         <v>1484</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="F3">
         <v>30</v>
@@ -10289,7 +10298,7 @@
         <v>16422</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.29920000000000002</v>
       </c>
       <c r="F4">
         <v>30</v>
@@ -10309,7 +10318,7 @@
         <v>165063</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1.5295000000000001</v>
       </c>
       <c r="F5">
         <v>30</v>
@@ -10329,7 +10338,7 @@
         <v>1668222</v>
       </c>
       <c r="E6">
-        <v>12</v>
+        <v>7.6212999999999997</v>
       </c>
       <c r="F6">
         <v>30</v>
@@ -10349,7 +10358,7 @@
         <v>16645094</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>18.145</v>
       </c>
       <c r="F7">
         <v>30</v>
@@ -10369,7 +10378,7 @@
         <v>166528644</v>
       </c>
       <c r="E8">
-        <v>86</v>
+        <v>85.171000000000006</v>
       </c>
       <c r="F8">
         <v>30</v>
@@ -10389,7 +10398,7 @@
         <v>1664246688</v>
       </c>
       <c r="E9">
-        <v>1445</v>
+        <v>1364.43</v>
       </c>
       <c r="F9">
         <v>30</v>
@@ -10441,16 +10450,16 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>602</v>
+        <v>590</v>
       </c>
       <c r="C2">
-        <v>636</v>
+        <v>621</v>
       </c>
       <c r="D2">
-        <v>1238</v>
+        <v>1211</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>1.468</v>
       </c>
       <c r="F2">
         <v>42</v>
@@ -10461,16 +10470,16 @@
         <v>100</v>
       </c>
       <c r="B3">
-        <v>5161</v>
+        <v>5223</v>
       </c>
       <c r="C3">
-        <v>5571</v>
+        <v>5653</v>
       </c>
       <c r="D3">
-        <v>10732</v>
+        <v>10876</v>
       </c>
       <c r="E3">
-        <v>9</v>
+        <v>8.3978999999999999</v>
       </c>
       <c r="F3">
         <v>42</v>
@@ -10481,16 +10490,16 @@
         <v>1000</v>
       </c>
       <c r="B4">
-        <v>38908</v>
+        <v>38855</v>
       </c>
       <c r="C4">
-        <v>43372</v>
+        <v>43304</v>
       </c>
       <c r="D4">
-        <v>82280</v>
+        <v>82159</v>
       </c>
       <c r="E4">
-        <v>13</v>
+        <v>14.143800000000001</v>
       </c>
       <c r="F4">
         <v>42</v>
@@ -10501,16 +10510,16 @@
         <v>10000</v>
       </c>
       <c r="B5">
-        <v>306706</v>
+        <v>306877</v>
       </c>
       <c r="C5">
-        <v>353275</v>
+        <v>353661</v>
       </c>
       <c r="D5">
-        <v>659981</v>
+        <v>660538</v>
       </c>
       <c r="E5">
-        <v>58</v>
+        <v>57.830399999999997</v>
       </c>
       <c r="F5">
         <v>42</v>
@@ -10521,16 +10530,16 @@
         <v>100000</v>
       </c>
       <c r="B6">
-        <v>2564239</v>
+        <v>2563768</v>
       </c>
       <c r="C6">
-        <v>3037738</v>
+        <v>3037318</v>
       </c>
       <c r="D6">
-        <v>5601977</v>
+        <v>5601086</v>
       </c>
       <c r="E6">
-        <v>255</v>
+        <v>243.4845</v>
       </c>
       <c r="F6">
         <v>42</v>
@@ -10541,16 +10550,16 @@
         <v>1000000</v>
       </c>
       <c r="B7">
-        <v>22195895</v>
+        <v>22192347</v>
       </c>
       <c r="C7">
-        <v>26822389</v>
+        <v>26816993</v>
       </c>
       <c r="D7">
-        <v>49018284</v>
+        <v>49009340</v>
       </c>
       <c r="E7">
-        <v>2307</v>
+        <v>1482.2955999999999</v>
       </c>
       <c r="F7">
         <v>42</v>
@@ -10561,16 +10570,16 @@
         <v>10000000</v>
       </c>
       <c r="B8">
-        <v>199880323</v>
+        <v>199879872</v>
       </c>
       <c r="C8">
-        <v>247165471</v>
+        <v>247163424</v>
       </c>
       <c r="D8">
-        <v>447045794</v>
+        <v>447043296</v>
       </c>
       <c r="E8">
-        <v>19675</v>
+        <v>12684.3938</v>
       </c>
       <c r="F8">
         <v>42</v>
@@ -10581,16 +10590,16 @@
         <v>100000000</v>
       </c>
       <c r="B9">
-        <v>1830373607</v>
+        <v>1830361328</v>
       </c>
       <c r="C9">
-        <v>2304561056</v>
+        <v>2304541680</v>
       </c>
       <c r="D9">
-        <v>4134934663</v>
+        <v>4134903008</v>
       </c>
       <c r="E9">
-        <v>193228</v>
+        <v>119225.60649999999</v>
       </c>
       <c r="F9">
         <v>42</v>

</xml_diff>